<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@58792fd0c65ea066198dde2ae7a1c86386392610 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-AdvanceDirective.xlsx
+++ b/StructureDefinition-AdvanceDirective.xlsx
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-08-06T09:01:08+00:00</t>
+    <t>2024-08-06T13:05:08+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@6d2b3232d5d87fd42b4f97f2958f1ce115184c05 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-AdvanceDirective.xlsx
+++ b/StructureDefinition-AdvanceDirective.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.12.0</t>
+    <t>1.13.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-18T10:21:48+00:00</t>
+    <t>2025-03-18T10:31:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@e358b7a546714077bc6eddd637cae2f46dcd7870 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-AdvanceDirective.xlsx
+++ b/StructureDefinition-AdvanceDirective.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.13.0</t>
+    <t>1.14.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-01T10:36:45+00:00</t>
+    <t>2025-04-01T10:40:06+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>